<commit_message>
ci: make e2e-test-pipeline and all test runners bulletproof with zero errors and artifact downloads
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/StainScope_Security_Test_Report.xlsx
+++ b/Vulnerability Test Results/StainScope_Security_Test_Report.xlsx
@@ -189,7 +189,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-08-21 08:35:43</t>
+    <t>2026-08-21 09:23:00</t>
   </si>
   <si>
     <t>TC002</t>
@@ -5594,7 +5594,6 @@
     <col min="6" max="7" width="42" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5655,7 +5654,7 @@
         <v>56</v>
       </c>
       <c r="I2" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J2" s="16" t="s">
         <v>57</v>
@@ -5687,7 +5686,7 @@
         <v>56</v>
       </c>
       <c r="I3" s="18">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J3" s="18" t="s">
         <v>57</v>
@@ -5751,7 +5750,7 @@
         <v>56</v>
       </c>
       <c r="I5" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J5" s="18" t="s">
         <v>57</v>
@@ -5783,7 +5782,7 @@
         <v>56</v>
       </c>
       <c r="I6" s="16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J6" s="16" t="s">
         <v>57</v>
@@ -5815,7 +5814,7 @@
         <v>56</v>
       </c>
       <c r="I7" s="18">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J7" s="18" t="s">
         <v>57</v>
@@ -5847,7 +5846,7 @@
         <v>56</v>
       </c>
       <c r="I8" s="16">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J8" s="16" t="s">
         <v>57</v>
@@ -5975,7 +5974,7 @@
         <v>56</v>
       </c>
       <c r="I12" s="16">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J12" s="16" t="s">
         <v>57</v>
@@ -6007,7 +6006,7 @@
         <v>56</v>
       </c>
       <c r="I13" s="18">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J13" s="18" t="s">
         <v>57</v>
@@ -6039,7 +6038,7 @@
         <v>56</v>
       </c>
       <c r="I14" s="16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>57</v>
@@ -6103,7 +6102,7 @@
         <v>56</v>
       </c>
       <c r="I16" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>57</v>
@@ -6135,7 +6134,7 @@
         <v>56</v>
       </c>
       <c r="I17" s="18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J17" s="18" t="s">
         <v>57</v>
@@ -6167,7 +6166,7 @@
         <v>56</v>
       </c>
       <c r="I18" s="16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J18" s="16" t="s">
         <v>57</v>
@@ -6199,7 +6198,7 @@
         <v>56</v>
       </c>
       <c r="I19" s="18">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J19" s="18" t="s">
         <v>57</v>
@@ -6231,7 +6230,7 @@
         <v>56</v>
       </c>
       <c r="I20" s="16">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>57</v>
@@ -6263,7 +6262,7 @@
         <v>56</v>
       </c>
       <c r="I21" s="18">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J21" s="18" t="s">
         <v>57</v>
@@ -6295,7 +6294,7 @@
         <v>56</v>
       </c>
       <c r="I22" s="16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>57</v>
@@ -6327,7 +6326,7 @@
         <v>56</v>
       </c>
       <c r="I23" s="18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J23" s="18" t="s">
         <v>57</v>
@@ -6359,7 +6358,7 @@
         <v>56</v>
       </c>
       <c r="I24" s="16">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J24" s="16" t="s">
         <v>57</v>
@@ -6391,7 +6390,7 @@
         <v>56</v>
       </c>
       <c r="I25" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J25" s="18" t="s">
         <v>57</v>
@@ -6423,7 +6422,7 @@
         <v>56</v>
       </c>
       <c r="I26" s="16">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J26" s="16" t="s">
         <v>57</v>
@@ -6455,7 +6454,7 @@
         <v>56</v>
       </c>
       <c r="I27" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J27" s="18" t="s">
         <v>57</v>
@@ -6487,7 +6486,7 @@
         <v>56</v>
       </c>
       <c r="I28" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J28" s="16" t="s">
         <v>57</v>
@@ -6519,7 +6518,7 @@
         <v>56</v>
       </c>
       <c r="I29" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J29" s="18" t="s">
         <v>57</v>
@@ -6551,7 +6550,7 @@
         <v>56</v>
       </c>
       <c r="I30" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J30" s="16" t="s">
         <v>57</v>
@@ -6583,7 +6582,7 @@
         <v>56</v>
       </c>
       <c r="I31" s="18">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J31" s="18" t="s">
         <v>57</v>
@@ -6615,7 +6614,7 @@
         <v>56</v>
       </c>
       <c r="I32" s="16">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>57</v>
@@ -6647,7 +6646,7 @@
         <v>56</v>
       </c>
       <c r="I33" s="18">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J33" s="18" t="s">
         <v>57</v>
@@ -6679,7 +6678,7 @@
         <v>56</v>
       </c>
       <c r="I34" s="16">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J34" s="16" t="s">
         <v>57</v>
@@ -6711,7 +6710,7 @@
         <v>56</v>
       </c>
       <c r="I35" s="18">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J35" s="18" t="s">
         <v>57</v>
@@ -6743,7 +6742,7 @@
         <v>56</v>
       </c>
       <c r="I36" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J36" s="16" t="s">
         <v>57</v>
@@ -6775,7 +6774,7 @@
         <v>56</v>
       </c>
       <c r="I37" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J37" s="18" t="s">
         <v>57</v>
@@ -6807,7 +6806,7 @@
         <v>56</v>
       </c>
       <c r="I38" s="16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J38" s="16" t="s">
         <v>57</v>
@@ -6839,7 +6838,7 @@
         <v>56</v>
       </c>
       <c r="I39" s="18">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J39" s="18" t="s">
         <v>57</v>
@@ -6871,7 +6870,7 @@
         <v>56</v>
       </c>
       <c r="I40" s="16">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J40" s="16" t="s">
         <v>57</v>
@@ -6903,7 +6902,7 @@
         <v>56</v>
       </c>
       <c r="I41" s="18">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J41" s="18" t="s">
         <v>57</v>
@@ -6935,7 +6934,7 @@
         <v>56</v>
       </c>
       <c r="I42" s="16">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J42" s="16" t="s">
         <v>57</v>
@@ -6967,7 +6966,7 @@
         <v>56</v>
       </c>
       <c r="I43" s="18">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J43" s="18" t="s">
         <v>57</v>
@@ -6999,7 +6998,7 @@
         <v>56</v>
       </c>
       <c r="I44" s="16">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J44" s="16" t="s">
         <v>57</v>
@@ -7031,7 +7030,7 @@
         <v>56</v>
       </c>
       <c r="I45" s="18">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J45" s="18" t="s">
         <v>57</v>
@@ -7063,7 +7062,7 @@
         <v>56</v>
       </c>
       <c r="I46" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J46" s="16" t="s">
         <v>57</v>
@@ -7127,7 +7126,7 @@
         <v>56</v>
       </c>
       <c r="I48" s="16">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J48" s="16" t="s">
         <v>57</v>
@@ -7159,7 +7158,7 @@
         <v>56</v>
       </c>
       <c r="I49" s="18">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J49" s="18" t="s">
         <v>57</v>
@@ -7191,7 +7190,7 @@
         <v>56</v>
       </c>
       <c r="I50" s="16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J50" s="16" t="s">
         <v>57</v>
@@ -7223,7 +7222,7 @@
         <v>56</v>
       </c>
       <c r="I51" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J51" s="18" t="s">
         <v>57</v>
@@ -7255,7 +7254,7 @@
         <v>56</v>
       </c>
       <c r="I52" s="16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J52" s="16" t="s">
         <v>57</v>
@@ -7287,7 +7286,7 @@
         <v>56</v>
       </c>
       <c r="I53" s="18">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J53" s="18" t="s">
         <v>57</v>
@@ -7319,7 +7318,7 @@
         <v>56</v>
       </c>
       <c r="I54" s="16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J54" s="16" t="s">
         <v>57</v>
@@ -7383,7 +7382,7 @@
         <v>56</v>
       </c>
       <c r="I56" s="16">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J56" s="16" t="s">
         <v>57</v>
@@ -7415,7 +7414,7 @@
         <v>56</v>
       </c>
       <c r="I57" s="18">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J57" s="18" t="s">
         <v>57</v>
@@ -7447,7 +7446,7 @@
         <v>56</v>
       </c>
       <c r="I58" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J58" s="16" t="s">
         <v>57</v>
@@ -7479,7 +7478,7 @@
         <v>56</v>
       </c>
       <c r="I59" s="18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J59" s="18" t="s">
         <v>57</v>
@@ -7511,7 +7510,7 @@
         <v>56</v>
       </c>
       <c r="I60" s="16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J60" s="16" t="s">
         <v>57</v>
@@ -7575,7 +7574,7 @@
         <v>56</v>
       </c>
       <c r="I62" s="16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J62" s="16" t="s">
         <v>57</v>
@@ -7607,7 +7606,7 @@
         <v>56</v>
       </c>
       <c r="I63" s="18">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J63" s="18" t="s">
         <v>57</v>
@@ -7639,7 +7638,7 @@
         <v>56</v>
       </c>
       <c r="I64" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J64" s="16" t="s">
         <v>57</v>
@@ -7671,7 +7670,7 @@
         <v>56</v>
       </c>
       <c r="I65" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J65" s="18" t="s">
         <v>57</v>
@@ -7703,7 +7702,7 @@
         <v>56</v>
       </c>
       <c r="I66" s="16">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J66" s="16" t="s">
         <v>57</v>
@@ -7735,7 +7734,7 @@
         <v>56</v>
       </c>
       <c r="I67" s="18">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J67" s="18" t="s">
         <v>57</v>
@@ -7799,7 +7798,7 @@
         <v>56</v>
       </c>
       <c r="I69" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J69" s="18" t="s">
         <v>57</v>
@@ -7831,7 +7830,7 @@
         <v>56</v>
       </c>
       <c r="I70" s="16">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J70" s="16" t="s">
         <v>57</v>
@@ -7863,7 +7862,7 @@
         <v>56</v>
       </c>
       <c r="I71" s="18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J71" s="18" t="s">
         <v>57</v>
@@ -7895,7 +7894,7 @@
         <v>56</v>
       </c>
       <c r="I72" s="16">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J72" s="16" t="s">
         <v>57</v>
@@ -7927,7 +7926,7 @@
         <v>56</v>
       </c>
       <c r="I73" s="18">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J73" s="18" t="s">
         <v>57</v>
@@ -7959,7 +7958,7 @@
         <v>56</v>
       </c>
       <c r="I74" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J74" s="16" t="s">
         <v>57</v>
@@ -7991,7 +7990,7 @@
         <v>56</v>
       </c>
       <c r="I75" s="18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J75" s="18" t="s">
         <v>57</v>
@@ -8023,7 +8022,7 @@
         <v>56</v>
       </c>
       <c r="I76" s="16">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J76" s="16" t="s">
         <v>57</v>
@@ -8055,7 +8054,7 @@
         <v>56</v>
       </c>
       <c r="I77" s="18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J77" s="18" t="s">
         <v>57</v>
@@ -8087,7 +8086,7 @@
         <v>56</v>
       </c>
       <c r="I78" s="16">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J78" s="16" t="s">
         <v>57</v>
@@ -8119,7 +8118,7 @@
         <v>56</v>
       </c>
       <c r="I79" s="18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J79" s="18" t="s">
         <v>57</v>
@@ -8151,7 +8150,7 @@
         <v>56</v>
       </c>
       <c r="I80" s="16">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J80" s="16" t="s">
         <v>57</v>
@@ -8183,7 +8182,7 @@
         <v>56</v>
       </c>
       <c r="I81" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J81" s="18" t="s">
         <v>57</v>
@@ -8215,7 +8214,7 @@
         <v>56</v>
       </c>
       <c r="I82" s="16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J82" s="16" t="s">
         <v>57</v>
@@ -8247,7 +8246,7 @@
         <v>56</v>
       </c>
       <c r="I83" s="18">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J83" s="18" t="s">
         <v>57</v>
@@ -8279,7 +8278,7 @@
         <v>56</v>
       </c>
       <c r="I84" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J84" s="16" t="s">
         <v>57</v>
@@ -8311,7 +8310,7 @@
         <v>56</v>
       </c>
       <c r="I85" s="18">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J85" s="18" t="s">
         <v>57</v>
@@ -8343,7 +8342,7 @@
         <v>56</v>
       </c>
       <c r="I86" s="16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J86" s="16" t="s">
         <v>57</v>
@@ -8375,7 +8374,7 @@
         <v>56</v>
       </c>
       <c r="I87" s="18">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J87" s="18" t="s">
         <v>57</v>
@@ -8407,7 +8406,7 @@
         <v>56</v>
       </c>
       <c r="I88" s="16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J88" s="16" t="s">
         <v>57</v>
@@ -8439,7 +8438,7 @@
         <v>56</v>
       </c>
       <c r="I89" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J89" s="18" t="s">
         <v>57</v>
@@ -8471,7 +8470,7 @@
         <v>56</v>
       </c>
       <c r="I90" s="16">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J90" s="16" t="s">
         <v>57</v>
@@ -8503,7 +8502,7 @@
         <v>56</v>
       </c>
       <c r="I91" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J91" s="18" t="s">
         <v>57</v>
@@ -8535,7 +8534,7 @@
         <v>56</v>
       </c>
       <c r="I92" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J92" s="16" t="s">
         <v>57</v>
@@ -8567,7 +8566,7 @@
         <v>56</v>
       </c>
       <c r="I93" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J93" s="18" t="s">
         <v>57</v>
@@ -8599,7 +8598,7 @@
         <v>56</v>
       </c>
       <c r="I94" s="16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J94" s="16" t="s">
         <v>57</v>
@@ -8631,7 +8630,7 @@
         <v>56</v>
       </c>
       <c r="I95" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J95" s="18" t="s">
         <v>57</v>
@@ -8663,7 +8662,7 @@
         <v>56</v>
       </c>
       <c r="I96" s="16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J96" s="16" t="s">
         <v>57</v>
@@ -8695,7 +8694,7 @@
         <v>56</v>
       </c>
       <c r="I97" s="18">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J97" s="18" t="s">
         <v>57</v>
@@ -8727,7 +8726,7 @@
         <v>56</v>
       </c>
       <c r="I98" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J98" s="16" t="s">
         <v>57</v>
@@ -8759,7 +8758,7 @@
         <v>56</v>
       </c>
       <c r="I99" s="18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J99" s="18" t="s">
         <v>57</v>
@@ -8791,7 +8790,7 @@
         <v>56</v>
       </c>
       <c r="I100" s="16">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J100" s="16" t="s">
         <v>57</v>
@@ -8855,7 +8854,7 @@
         <v>56</v>
       </c>
       <c r="I102" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J102" s="16" t="s">
         <v>57</v>
@@ -8887,7 +8886,7 @@
         <v>56</v>
       </c>
       <c r="I103" s="18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J103" s="18" t="s">
         <v>57</v>
@@ -8919,7 +8918,7 @@
         <v>56</v>
       </c>
       <c r="I104" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J104" s="16" t="s">
         <v>57</v>
@@ -8983,7 +8982,7 @@
         <v>56</v>
       </c>
       <c r="I106" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J106" s="16" t="s">
         <v>57</v>
@@ -9015,7 +9014,7 @@
         <v>56</v>
       </c>
       <c r="I107" s="18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J107" s="18" t="s">
         <v>57</v>
@@ -9047,7 +9046,7 @@
         <v>56</v>
       </c>
       <c r="I108" s="16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J108" s="16" t="s">
         <v>57</v>
@@ -9111,7 +9110,7 @@
         <v>56</v>
       </c>
       <c r="I110" s="16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J110" s="16" t="s">
         <v>57</v>
@@ -9175,7 +9174,7 @@
         <v>56</v>
       </c>
       <c r="I112" s="16">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J112" s="16" t="s">
         <v>57</v>
@@ -9207,7 +9206,7 @@
         <v>56</v>
       </c>
       <c r="I113" s="18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J113" s="18" t="s">
         <v>57</v>
@@ -9271,7 +9270,7 @@
         <v>56</v>
       </c>
       <c r="I115" s="18">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J115" s="18" t="s">
         <v>57</v>
@@ -9303,7 +9302,7 @@
         <v>56</v>
       </c>
       <c r="I116" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J116" s="16" t="s">
         <v>57</v>
@@ -9335,7 +9334,7 @@
         <v>56</v>
       </c>
       <c r="I117" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J117" s="18" t="s">
         <v>57</v>
@@ -9367,7 +9366,7 @@
         <v>56</v>
       </c>
       <c r="I118" s="16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J118" s="16" t="s">
         <v>57</v>
@@ -9399,7 +9398,7 @@
         <v>56</v>
       </c>
       <c r="I119" s="18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J119" s="18" t="s">
         <v>57</v>
@@ -9431,7 +9430,7 @@
         <v>56</v>
       </c>
       <c r="I120" s="16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J120" s="16" t="s">
         <v>57</v>
@@ -9463,7 +9462,7 @@
         <v>56</v>
       </c>
       <c r="I121" s="18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J121" s="18" t="s">
         <v>57</v>
@@ -9559,7 +9558,7 @@
         <v>56</v>
       </c>
       <c r="I124" s="16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J124" s="16" t="s">
         <v>57</v>
@@ -9591,7 +9590,7 @@
         <v>56</v>
       </c>
       <c r="I125" s="18">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J125" s="18" t="s">
         <v>57</v>
@@ -9655,7 +9654,7 @@
         <v>56</v>
       </c>
       <c r="I127" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J127" s="18" t="s">
         <v>57</v>
@@ -9687,7 +9686,7 @@
         <v>56</v>
       </c>
       <c r="I128" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J128" s="16" t="s">
         <v>57</v>
@@ -9719,7 +9718,7 @@
         <v>56</v>
       </c>
       <c r="I129" s="18">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J129" s="18" t="s">
         <v>57</v>
@@ -9751,7 +9750,7 @@
         <v>56</v>
       </c>
       <c r="I130" s="16">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J130" s="16" t="s">
         <v>57</v>
@@ -9783,7 +9782,7 @@
         <v>56</v>
       </c>
       <c r="I131" s="18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J131" s="18" t="s">
         <v>57</v>
@@ -9847,7 +9846,7 @@
         <v>56</v>
       </c>
       <c r="I133" s="18">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J133" s="18" t="s">
         <v>57</v>
@@ -9879,7 +9878,7 @@
         <v>56</v>
       </c>
       <c r="I134" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J134" s="16" t="s">
         <v>57</v>
@@ -9911,7 +9910,7 @@
         <v>56</v>
       </c>
       <c r="I135" s="18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J135" s="18" t="s">
         <v>57</v>
@@ -9943,7 +9942,7 @@
         <v>56</v>
       </c>
       <c r="I136" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J136" s="16" t="s">
         <v>57</v>
@@ -9975,7 +9974,7 @@
         <v>56</v>
       </c>
       <c r="I137" s="18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J137" s="18" t="s">
         <v>57</v>
@@ -10007,7 +10006,7 @@
         <v>56</v>
       </c>
       <c r="I138" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J138" s="16" t="s">
         <v>57</v>
@@ -10039,7 +10038,7 @@
         <v>56</v>
       </c>
       <c r="I139" s="18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J139" s="18" t="s">
         <v>57</v>
@@ -10071,7 +10070,7 @@
         <v>56</v>
       </c>
       <c r="I140" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J140" s="16" t="s">
         <v>57</v>
@@ -10103,7 +10102,7 @@
         <v>56</v>
       </c>
       <c r="I141" s="18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J141" s="18" t="s">
         <v>57</v>
@@ -10135,7 +10134,7 @@
         <v>56</v>
       </c>
       <c r="I142" s="16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J142" s="16" t="s">
         <v>57</v>
@@ -10167,7 +10166,7 @@
         <v>56</v>
       </c>
       <c r="I143" s="18">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J143" s="18" t="s">
         <v>57</v>
@@ -10199,7 +10198,7 @@
         <v>56</v>
       </c>
       <c r="I144" s="16">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J144" s="16" t="s">
         <v>57</v>
@@ -10263,7 +10262,7 @@
         <v>56</v>
       </c>
       <c r="I146" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J146" s="16" t="s">
         <v>57</v>
@@ -10295,7 +10294,7 @@
         <v>56</v>
       </c>
       <c r="I147" s="18">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J147" s="18" t="s">
         <v>57</v>
@@ -10327,7 +10326,7 @@
         <v>56</v>
       </c>
       <c r="I148" s="16">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J148" s="16" t="s">
         <v>57</v>
@@ -10359,7 +10358,7 @@
         <v>56</v>
       </c>
       <c r="I149" s="18">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J149" s="18" t="s">
         <v>57</v>
@@ -10391,7 +10390,7 @@
         <v>56</v>
       </c>
       <c r="I150" s="16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J150" s="16" t="s">
         <v>57</v>
@@ -10423,7 +10422,7 @@
         <v>56</v>
       </c>
       <c r="I151" s="18">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J151" s="18" t="s">
         <v>57</v>
@@ -10455,7 +10454,7 @@
         <v>56</v>
       </c>
       <c r="I152" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J152" s="16" t="s">
         <v>57</v>
@@ -10519,7 +10518,7 @@
         <v>56</v>
       </c>
       <c r="I154" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J154" s="16" t="s">
         <v>57</v>
@@ -10551,7 +10550,7 @@
         <v>56</v>
       </c>
       <c r="I155" s="18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J155" s="18" t="s">
         <v>57</v>
@@ -10583,7 +10582,7 @@
         <v>56</v>
       </c>
       <c r="I156" s="16">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J156" s="16" t="s">
         <v>57</v>
@@ -10647,7 +10646,7 @@
         <v>56</v>
       </c>
       <c r="I158" s="16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J158" s="16" t="s">
         <v>57</v>
@@ -10679,7 +10678,7 @@
         <v>56</v>
       </c>
       <c r="I159" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J159" s="18" t="s">
         <v>57</v>
@@ -10711,7 +10710,7 @@
         <v>56</v>
       </c>
       <c r="I160" s="16">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J160" s="16" t="s">
         <v>57</v>
@@ -10743,7 +10742,7 @@
         <v>56</v>
       </c>
       <c r="I161" s="18">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J161" s="18" t="s">
         <v>57</v>
@@ -10775,7 +10774,7 @@
         <v>56</v>
       </c>
       <c r="I162" s="16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J162" s="16" t="s">
         <v>57</v>
@@ -10807,7 +10806,7 @@
         <v>56</v>
       </c>
       <c r="I163" s="18">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J163" s="18" t="s">
         <v>57</v>
@@ -10839,7 +10838,7 @@
         <v>56</v>
       </c>
       <c r="I164" s="16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J164" s="16" t="s">
         <v>57</v>
@@ -10871,7 +10870,7 @@
         <v>56</v>
       </c>
       <c r="I165" s="18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J165" s="18" t="s">
         <v>57</v>
@@ -10903,7 +10902,7 @@
         <v>56</v>
       </c>
       <c r="I166" s="16">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J166" s="16" t="s">
         <v>57</v>
@@ -10935,7 +10934,7 @@
         <v>56</v>
       </c>
       <c r="I167" s="18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J167" s="18" t="s">
         <v>57</v>
@@ -10967,7 +10966,7 @@
         <v>56</v>
       </c>
       <c r="I168" s="16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J168" s="16" t="s">
         <v>57</v>
@@ -10999,7 +10998,7 @@
         <v>56</v>
       </c>
       <c r="I169" s="18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J169" s="18" t="s">
         <v>57</v>
@@ -11031,7 +11030,7 @@
         <v>56</v>
       </c>
       <c r="I170" s="16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J170" s="16" t="s">
         <v>57</v>
@@ -11095,7 +11094,7 @@
         <v>56</v>
       </c>
       <c r="I172" s="16">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J172" s="16" t="s">
         <v>57</v>
@@ -11159,7 +11158,7 @@
         <v>56</v>
       </c>
       <c r="I174" s="16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J174" s="16" t="s">
         <v>57</v>
@@ -11191,7 +11190,7 @@
         <v>56</v>
       </c>
       <c r="I175" s="18">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J175" s="18" t="s">
         <v>57</v>
@@ -11223,7 +11222,7 @@
         <v>56</v>
       </c>
       <c r="I176" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J176" s="16" t="s">
         <v>57</v>
@@ -11255,7 +11254,7 @@
         <v>56</v>
       </c>
       <c r="I177" s="18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J177" s="18" t="s">
         <v>57</v>
@@ -11287,7 +11286,7 @@
         <v>56</v>
       </c>
       <c r="I178" s="16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J178" s="16" t="s">
         <v>57</v>
@@ -11351,7 +11350,7 @@
         <v>56</v>
       </c>
       <c r="I180" s="16">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J180" s="16" t="s">
         <v>57</v>
@@ -11383,7 +11382,7 @@
         <v>56</v>
       </c>
       <c r="I181" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J181" s="18" t="s">
         <v>57</v>
@@ -11415,7 +11414,7 @@
         <v>56</v>
       </c>
       <c r="I182" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J182" s="16" t="s">
         <v>57</v>
@@ -11479,7 +11478,7 @@
         <v>56</v>
       </c>
       <c r="I184" s="16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J184" s="16" t="s">
         <v>57</v>
@@ -11511,7 +11510,7 @@
         <v>56</v>
       </c>
       <c r="I185" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J185" s="18" t="s">
         <v>57</v>
@@ -11543,7 +11542,7 @@
         <v>56</v>
       </c>
       <c r="I186" s="16">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J186" s="16" t="s">
         <v>57</v>
@@ -11575,7 +11574,7 @@
         <v>56</v>
       </c>
       <c r="I187" s="18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J187" s="18" t="s">
         <v>57</v>
@@ -11607,7 +11606,7 @@
         <v>56</v>
       </c>
       <c r="I188" s="16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J188" s="16" t="s">
         <v>57</v>
@@ -11639,7 +11638,7 @@
         <v>56</v>
       </c>
       <c r="I189" s="18">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J189" s="18" t="s">
         <v>57</v>
@@ -11671,7 +11670,7 @@
         <v>56</v>
       </c>
       <c r="I190" s="16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J190" s="16" t="s">
         <v>57</v>
@@ -11735,7 +11734,7 @@
         <v>56</v>
       </c>
       <c r="I192" s="16">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J192" s="16" t="s">
         <v>57</v>
@@ -11767,7 +11766,7 @@
         <v>56</v>
       </c>
       <c r="I193" s="18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J193" s="18" t="s">
         <v>57</v>
@@ -11799,7 +11798,7 @@
         <v>56</v>
       </c>
       <c r="I194" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J194" s="16" t="s">
         <v>57</v>
@@ -11831,7 +11830,7 @@
         <v>56</v>
       </c>
       <c r="I195" s="18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J195" s="18" t="s">
         <v>57</v>
@@ -11895,7 +11894,7 @@
         <v>56</v>
       </c>
       <c r="I197" s="18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J197" s="18" t="s">
         <v>57</v>
@@ -11927,7 +11926,7 @@
         <v>56</v>
       </c>
       <c r="I198" s="16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J198" s="16" t="s">
         <v>57</v>
@@ -11959,7 +11958,7 @@
         <v>56</v>
       </c>
       <c r="I199" s="18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J199" s="18" t="s">
         <v>57</v>
@@ -11991,7 +11990,7 @@
         <v>56</v>
       </c>
       <c r="I200" s="16">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J200" s="16" t="s">
         <v>57</v>
@@ -12023,7 +12022,7 @@
         <v>56</v>
       </c>
       <c r="I201" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J201" s="18" t="s">
         <v>57</v>
@@ -12055,7 +12054,7 @@
         <v>56</v>
       </c>
       <c r="I202" s="16">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J202" s="16" t="s">
         <v>57</v>
@@ -12087,7 +12086,7 @@
         <v>56</v>
       </c>
       <c r="I203" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J203" s="18" t="s">
         <v>57</v>
@@ -12119,7 +12118,7 @@
         <v>56</v>
       </c>
       <c r="I204" s="16">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J204" s="16" t="s">
         <v>57</v>
@@ -12151,7 +12150,7 @@
         <v>56</v>
       </c>
       <c r="I205" s="18">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J205" s="18" t="s">
         <v>57</v>
@@ -12183,7 +12182,7 @@
         <v>56</v>
       </c>
       <c r="I206" s="16">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J206" s="16" t="s">
         <v>57</v>
@@ -12215,7 +12214,7 @@
         <v>56</v>
       </c>
       <c r="I207" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J207" s="18" t="s">
         <v>57</v>
@@ -12247,7 +12246,7 @@
         <v>56</v>
       </c>
       <c r="I208" s="16">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J208" s="16" t="s">
         <v>57</v>
@@ -12279,7 +12278,7 @@
         <v>56</v>
       </c>
       <c r="I209" s="18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J209" s="18" t="s">
         <v>57</v>
@@ -12311,7 +12310,7 @@
         <v>56</v>
       </c>
       <c r="I210" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J210" s="16" t="s">
         <v>57</v>
@@ -12343,7 +12342,7 @@
         <v>56</v>
       </c>
       <c r="I211" s="18">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J211" s="18" t="s">
         <v>57</v>
@@ -12375,7 +12374,7 @@
         <v>56</v>
       </c>
       <c r="I212" s="16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J212" s="16" t="s">
         <v>57</v>
@@ -12407,7 +12406,7 @@
         <v>56</v>
       </c>
       <c r="I213" s="18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J213" s="18" t="s">
         <v>57</v>
@@ -12471,7 +12470,7 @@
         <v>56</v>
       </c>
       <c r="I215" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J215" s="18" t="s">
         <v>57</v>
@@ -12503,7 +12502,7 @@
         <v>56</v>
       </c>
       <c r="I216" s="16">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J216" s="16" t="s">
         <v>57</v>
@@ -12567,7 +12566,7 @@
         <v>56</v>
       </c>
       <c r="I218" s="16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J218" s="16" t="s">
         <v>57</v>
@@ -12631,7 +12630,7 @@
         <v>56</v>
       </c>
       <c r="I220" s="16">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J220" s="16" t="s">
         <v>57</v>
@@ -12663,7 +12662,7 @@
         <v>56</v>
       </c>
       <c r="I221" s="18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J221" s="18" t="s">
         <v>57</v>
@@ -12727,7 +12726,7 @@
         <v>56</v>
       </c>
       <c r="I223" s="18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J223" s="18" t="s">
         <v>57</v>
@@ -12759,7 +12758,7 @@
         <v>56</v>
       </c>
       <c r="I224" s="16">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J224" s="16" t="s">
         <v>57</v>
@@ -12791,7 +12790,7 @@
         <v>56</v>
       </c>
       <c r="I225" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J225" s="18" t="s">
         <v>57</v>
@@ -12823,7 +12822,7 @@
         <v>56</v>
       </c>
       <c r="I226" s="16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J226" s="16" t="s">
         <v>57</v>
@@ -12855,7 +12854,7 @@
         <v>56</v>
       </c>
       <c r="I227" s="18">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J227" s="18" t="s">
         <v>57</v>
@@ -12887,7 +12886,7 @@
         <v>56</v>
       </c>
       <c r="I228" s="16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J228" s="16" t="s">
         <v>57</v>
@@ -12919,7 +12918,7 @@
         <v>56</v>
       </c>
       <c r="I229" s="18">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J229" s="18" t="s">
         <v>57</v>
@@ -12951,7 +12950,7 @@
         <v>56</v>
       </c>
       <c r="I230" s="16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J230" s="16" t="s">
         <v>57</v>
@@ -12983,7 +12982,7 @@
         <v>56</v>
       </c>
       <c r="I231" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J231" s="18" t="s">
         <v>57</v>
@@ -13015,7 +13014,7 @@
         <v>56</v>
       </c>
       <c r="I232" s="16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J232" s="16" t="s">
         <v>57</v>
@@ -13047,7 +13046,7 @@
         <v>56</v>
       </c>
       <c r="I233" s="18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J233" s="18" t="s">
         <v>57</v>
@@ -13079,7 +13078,7 @@
         <v>56</v>
       </c>
       <c r="I234" s="16">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J234" s="16" t="s">
         <v>57</v>
@@ -13111,7 +13110,7 @@
         <v>56</v>
       </c>
       <c r="I235" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J235" s="18" t="s">
         <v>57</v>
@@ -13175,7 +13174,7 @@
         <v>56</v>
       </c>
       <c r="I237" s="18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J237" s="18" t="s">
         <v>57</v>
@@ -13207,7 +13206,7 @@
         <v>56</v>
       </c>
       <c r="I238" s="16">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J238" s="16" t="s">
         <v>57</v>
@@ -13239,7 +13238,7 @@
         <v>56</v>
       </c>
       <c r="I239" s="18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J239" s="18" t="s">
         <v>57</v>
@@ -13271,7 +13270,7 @@
         <v>56</v>
       </c>
       <c r="I240" s="16">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J240" s="16" t="s">
         <v>57</v>
@@ -13303,7 +13302,7 @@
         <v>56</v>
       </c>
       <c r="I241" s="18">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J241" s="18" t="s">
         <v>57</v>
@@ -13335,7 +13334,7 @@
         <v>56</v>
       </c>
       <c r="I242" s="16">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J242" s="16" t="s">
         <v>57</v>
@@ -13399,7 +13398,7 @@
         <v>56</v>
       </c>
       <c r="I244" s="16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J244" s="16" t="s">
         <v>57</v>
@@ -13431,7 +13430,7 @@
         <v>56</v>
       </c>
       <c r="I245" s="18">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J245" s="18" t="s">
         <v>57</v>
@@ -13463,7 +13462,7 @@
         <v>56</v>
       </c>
       <c r="I246" s="16">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J246" s="16" t="s">
         <v>57</v>
@@ -13527,7 +13526,7 @@
         <v>56</v>
       </c>
       <c r="I248" s="16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J248" s="16" t="s">
         <v>57</v>
@@ -13559,7 +13558,7 @@
         <v>56</v>
       </c>
       <c r="I249" s="18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J249" s="18" t="s">
         <v>57</v>
@@ -13591,7 +13590,7 @@
         <v>56</v>
       </c>
       <c r="I250" s="16">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J250" s="16" t="s">
         <v>57</v>
@@ -13623,7 +13622,7 @@
         <v>56</v>
       </c>
       <c r="I251" s="18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J251" s="18" t="s">
         <v>57</v>
@@ -13655,7 +13654,7 @@
         <v>56</v>
       </c>
       <c r="I252" s="16">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J252" s="16" t="s">
         <v>57</v>
@@ -13687,7 +13686,7 @@
         <v>56</v>
       </c>
       <c r="I253" s="18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J253" s="18" t="s">
         <v>57</v>
@@ -13719,7 +13718,7 @@
         <v>56</v>
       </c>
       <c r="I254" s="16">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J254" s="16" t="s">
         <v>57</v>
@@ -13751,7 +13750,7 @@
         <v>56</v>
       </c>
       <c r="I255" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J255" s="18" t="s">
         <v>57</v>
@@ -13815,7 +13814,7 @@
         <v>56</v>
       </c>
       <c r="I257" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J257" s="18" t="s">
         <v>57</v>
@@ -13847,7 +13846,7 @@
         <v>56</v>
       </c>
       <c r="I258" s="16">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J258" s="16" t="s">
         <v>57</v>
@@ -13879,7 +13878,7 @@
         <v>56</v>
       </c>
       <c r="I259" s="18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J259" s="18" t="s">
         <v>57</v>
@@ -13943,7 +13942,7 @@
         <v>56</v>
       </c>
       <c r="I261" s="18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J261" s="18" t="s">
         <v>57</v>
@@ -13975,7 +13974,7 @@
         <v>56</v>
       </c>
       <c r="I262" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J262" s="16" t="s">
         <v>57</v>
@@ -14007,7 +14006,7 @@
         <v>56</v>
       </c>
       <c r="I263" s="18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J263" s="18" t="s">
         <v>57</v>
@@ -14039,7 +14038,7 @@
         <v>56</v>
       </c>
       <c r="I264" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J264" s="16" t="s">
         <v>57</v>
@@ -14071,7 +14070,7 @@
         <v>56</v>
       </c>
       <c r="I265" s="18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J265" s="18" t="s">
         <v>57</v>
@@ -14103,7 +14102,7 @@
         <v>56</v>
       </c>
       <c r="I266" s="16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J266" s="16" t="s">
         <v>57</v>
@@ -14135,7 +14134,7 @@
         <v>56</v>
       </c>
       <c r="I267" s="18">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J267" s="18" t="s">
         <v>57</v>
@@ -14167,7 +14166,7 @@
         <v>56</v>
       </c>
       <c r="I268" s="16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J268" s="16" t="s">
         <v>57</v>
@@ -14199,7 +14198,7 @@
         <v>56</v>
       </c>
       <c r="I269" s="18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J269" s="18" t="s">
         <v>57</v>
@@ -14263,7 +14262,7 @@
         <v>56</v>
       </c>
       <c r="I271" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J271" s="18" t="s">
         <v>57</v>
@@ -14295,7 +14294,7 @@
         <v>56</v>
       </c>
       <c r="I272" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J272" s="16" t="s">
         <v>57</v>
@@ -14327,7 +14326,7 @@
         <v>56</v>
       </c>
       <c r="I273" s="18">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J273" s="18" t="s">
         <v>57</v>
@@ -14359,7 +14358,7 @@
         <v>56</v>
       </c>
       <c r="I274" s="16">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J274" s="16" t="s">
         <v>57</v>
@@ -14391,7 +14390,7 @@
         <v>56</v>
       </c>
       <c r="I275" s="18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J275" s="18" t="s">
         <v>57</v>
@@ -14423,7 +14422,7 @@
         <v>56</v>
       </c>
       <c r="I276" s="16">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J276" s="16" t="s">
         <v>57</v>
@@ -14455,7 +14454,7 @@
         <v>56</v>
       </c>
       <c r="I277" s="18">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J277" s="18" t="s">
         <v>57</v>
@@ -14487,7 +14486,7 @@
         <v>56</v>
       </c>
       <c r="I278" s="16">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J278" s="16" t="s">
         <v>57</v>
@@ -14519,7 +14518,7 @@
         <v>56</v>
       </c>
       <c r="I279" s="18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J279" s="18" t="s">
         <v>57</v>
@@ -14551,7 +14550,7 @@
         <v>56</v>
       </c>
       <c r="I280" s="16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J280" s="16" t="s">
         <v>57</v>
@@ -14647,7 +14646,7 @@
         <v>56</v>
       </c>
       <c r="I283" s="18">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J283" s="18" t="s">
         <v>57</v>
@@ -14679,7 +14678,7 @@
         <v>56</v>
       </c>
       <c r="I284" s="16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J284" s="16" t="s">
         <v>57</v>
@@ -14711,7 +14710,7 @@
         <v>56</v>
       </c>
       <c r="I285" s="18">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J285" s="18" t="s">
         <v>57</v>
@@ -14743,7 +14742,7 @@
         <v>56</v>
       </c>
       <c r="I286" s="16">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J286" s="16" t="s">
         <v>57</v>
@@ -14871,7 +14870,7 @@
         <v>56</v>
       </c>
       <c r="I290" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J290" s="16" t="s">
         <v>57</v>
@@ -14903,7 +14902,7 @@
         <v>56</v>
       </c>
       <c r="I291" s="18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J291" s="18" t="s">
         <v>57</v>
@@ -14935,7 +14934,7 @@
         <v>56</v>
       </c>
       <c r="I292" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J292" s="16" t="s">
         <v>57</v>
@@ -14967,7 +14966,7 @@
         <v>56</v>
       </c>
       <c r="I293" s="18">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J293" s="18" t="s">
         <v>57</v>
@@ -14999,7 +14998,7 @@
         <v>56</v>
       </c>
       <c r="I294" s="16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J294" s="16" t="s">
         <v>57</v>
@@ -15031,7 +15030,7 @@
         <v>56</v>
       </c>
       <c r="I295" s="18">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J295" s="18" t="s">
         <v>57</v>
@@ -15063,7 +15062,7 @@
         <v>56</v>
       </c>
       <c r="I296" s="16">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J296" s="16" t="s">
         <v>57</v>
@@ -15095,7 +15094,7 @@
         <v>56</v>
       </c>
       <c r="I297" s="18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J297" s="18" t="s">
         <v>57</v>
@@ -15127,7 +15126,7 @@
         <v>56</v>
       </c>
       <c r="I298" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J298" s="16" t="s">
         <v>57</v>
@@ -15159,7 +15158,7 @@
         <v>56</v>
       </c>
       <c r="I299" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J299" s="18" t="s">
         <v>57</v>
@@ -15191,7 +15190,7 @@
         <v>56</v>
       </c>
       <c r="I300" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J300" s="16" t="s">
         <v>57</v>
@@ -15223,7 +15222,7 @@
         <v>56</v>
       </c>
       <c r="I301" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J301" s="18" t="s">
         <v>57</v>
@@ -15255,7 +15254,7 @@
         <v>56</v>
       </c>
       <c r="I302" s="16">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J302" s="16" t="s">
         <v>57</v>
@@ -15287,7 +15286,7 @@
         <v>56</v>
       </c>
       <c r="I303" s="18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J303" s="18" t="s">
         <v>57</v>
@@ -15319,7 +15318,7 @@
         <v>56</v>
       </c>
       <c r="I304" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J304" s="16" t="s">
         <v>57</v>
@@ -15351,7 +15350,7 @@
         <v>56</v>
       </c>
       <c r="I305" s="18">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J305" s="18" t="s">
         <v>57</v>
@@ -15383,7 +15382,7 @@
         <v>56</v>
       </c>
       <c r="I306" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J306" s="16" t="s">
         <v>57</v>
@@ -15415,7 +15414,7 @@
         <v>56</v>
       </c>
       <c r="I307" s="18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J307" s="18" t="s">
         <v>57</v>
@@ -15447,7 +15446,7 @@
         <v>56</v>
       </c>
       <c r="I308" s="16">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J308" s="16" t="s">
         <v>57</v>
@@ -15479,7 +15478,7 @@
         <v>56</v>
       </c>
       <c r="I309" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J309" s="18" t="s">
         <v>57</v>
@@ -15511,7 +15510,7 @@
         <v>56</v>
       </c>
       <c r="I310" s="16">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J310" s="16" t="s">
         <v>57</v>
@@ -15543,7 +15542,7 @@
         <v>56</v>
       </c>
       <c r="I311" s="18">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J311" s="18" t="s">
         <v>57</v>
@@ -15575,7 +15574,7 @@
         <v>56</v>
       </c>
       <c r="I312" s="16">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J312" s="16" t="s">
         <v>57</v>
@@ -15607,7 +15606,7 @@
         <v>56</v>
       </c>
       <c r="I313" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J313" s="18" t="s">
         <v>57</v>
@@ -15639,7 +15638,7 @@
         <v>56</v>
       </c>
       <c r="I314" s="16">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J314" s="16" t="s">
         <v>57</v>
@@ -15671,7 +15670,7 @@
         <v>56</v>
       </c>
       <c r="I315" s="18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J315" s="18" t="s">
         <v>57</v>
@@ -15703,7 +15702,7 @@
         <v>56</v>
       </c>
       <c r="I316" s="16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J316" s="16" t="s">
         <v>57</v>
@@ -15735,7 +15734,7 @@
         <v>56</v>
       </c>
       <c r="I317" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J317" s="18" t="s">
         <v>57</v>
@@ -15767,7 +15766,7 @@
         <v>56</v>
       </c>
       <c r="I318" s="16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J318" s="16" t="s">
         <v>57</v>
@@ -15799,7 +15798,7 @@
         <v>56</v>
       </c>
       <c r="I319" s="18">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J319" s="18" t="s">
         <v>57</v>
@@ -15831,7 +15830,7 @@
         <v>56</v>
       </c>
       <c r="I320" s="16">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J320" s="16" t="s">
         <v>57</v>
@@ -15863,7 +15862,7 @@
         <v>56</v>
       </c>
       <c r="I321" s="18">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J321" s="18" t="s">
         <v>57</v>
@@ -15895,7 +15894,7 @@
         <v>56</v>
       </c>
       <c r="I322" s="16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J322" s="16" t="s">
         <v>57</v>
@@ -15927,7 +15926,7 @@
         <v>56</v>
       </c>
       <c r="I323" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J323" s="18" t="s">
         <v>57</v>
@@ -15959,7 +15958,7 @@
         <v>56</v>
       </c>
       <c r="I324" s="16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J324" s="16" t="s">
         <v>57</v>
@@ -15991,7 +15990,7 @@
         <v>56</v>
       </c>
       <c r="I325" s="18">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J325" s="18" t="s">
         <v>57</v>
@@ -16023,7 +16022,7 @@
         <v>56</v>
       </c>
       <c r="I326" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J326" s="16" t="s">
         <v>57</v>
@@ -16055,7 +16054,7 @@
         <v>56</v>
       </c>
       <c r="I327" s="18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J327" s="18" t="s">
         <v>57</v>
@@ -16087,7 +16086,7 @@
         <v>56</v>
       </c>
       <c r="I328" s="16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J328" s="16" t="s">
         <v>57</v>
@@ -16119,7 +16118,7 @@
         <v>56</v>
       </c>
       <c r="I329" s="18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J329" s="18" t="s">
         <v>57</v>
@@ -16151,7 +16150,7 @@
         <v>56</v>
       </c>
       <c r="I330" s="16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J330" s="16" t="s">
         <v>57</v>
@@ -16183,7 +16182,7 @@
         <v>56</v>
       </c>
       <c r="I331" s="18">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J331" s="18" t="s">
         <v>57</v>
@@ -16215,7 +16214,7 @@
         <v>56</v>
       </c>
       <c r="I332" s="16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J332" s="16" t="s">
         <v>57</v>
@@ -16247,7 +16246,7 @@
         <v>56</v>
       </c>
       <c r="I333" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J333" s="18" t="s">
         <v>57</v>
@@ -16279,7 +16278,7 @@
         <v>56</v>
       </c>
       <c r="I334" s="16">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J334" s="16" t="s">
         <v>57</v>
@@ -16311,7 +16310,7 @@
         <v>56</v>
       </c>
       <c r="I335" s="18">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J335" s="18" t="s">
         <v>57</v>
@@ -16343,7 +16342,7 @@
         <v>56</v>
       </c>
       <c r="I336" s="16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J336" s="16" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
chore: unify all CI pipelines exclusively into e2e-test-pipeline
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/StainScope_Security_Test_Report.xlsx
+++ b/Vulnerability Test Results/StainScope_Security_Test_Report.xlsx
@@ -189,7 +189,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-08-21 09:23:00</t>
+    <t>2026-08-21 09:28:01</t>
   </si>
   <si>
     <t>TC002</t>
@@ -5654,7 +5654,7 @@
         <v>56</v>
       </c>
       <c r="I2" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J2" s="16" t="s">
         <v>57</v>
@@ -5686,7 +5686,7 @@
         <v>56</v>
       </c>
       <c r="I3" s="18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J3" s="18" t="s">
         <v>57</v>
@@ -5718,7 +5718,7 @@
         <v>56</v>
       </c>
       <c r="I4" s="16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J4" s="16" t="s">
         <v>57</v>
@@ -5782,7 +5782,7 @@
         <v>56</v>
       </c>
       <c r="I6" s="16">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J6" s="16" t="s">
         <v>57</v>
@@ -5846,7 +5846,7 @@
         <v>56</v>
       </c>
       <c r="I8" s="16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J8" s="16" t="s">
         <v>57</v>
@@ -5878,7 +5878,7 @@
         <v>56</v>
       </c>
       <c r="I9" s="18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" s="18" t="s">
         <v>57</v>
@@ -5910,7 +5910,7 @@
         <v>56</v>
       </c>
       <c r="I10" s="16">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J10" s="16" t="s">
         <v>57</v>
@@ -5942,7 +5942,7 @@
         <v>56</v>
       </c>
       <c r="I11" s="18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J11" s="18" t="s">
         <v>57</v>
@@ -5974,7 +5974,7 @@
         <v>56</v>
       </c>
       <c r="I12" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J12" s="16" t="s">
         <v>57</v>
@@ -6006,7 +6006,7 @@
         <v>56</v>
       </c>
       <c r="I13" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13" s="18" t="s">
         <v>57</v>
@@ -6038,7 +6038,7 @@
         <v>56</v>
       </c>
       <c r="I14" s="16">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>57</v>
@@ -6070,7 +6070,7 @@
         <v>56</v>
       </c>
       <c r="I15" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J15" s="18" t="s">
         <v>57</v>
@@ -6102,7 +6102,7 @@
         <v>56</v>
       </c>
       <c r="I16" s="16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>57</v>
@@ -6134,7 +6134,7 @@
         <v>56</v>
       </c>
       <c r="I17" s="18">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J17" s="18" t="s">
         <v>57</v>
@@ -6166,7 +6166,7 @@
         <v>56</v>
       </c>
       <c r="I18" s="16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J18" s="16" t="s">
         <v>57</v>
@@ -6230,7 +6230,7 @@
         <v>56</v>
       </c>
       <c r="I20" s="16">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>57</v>
@@ -6262,7 +6262,7 @@
         <v>56</v>
       </c>
       <c r="I21" s="18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J21" s="18" t="s">
         <v>57</v>
@@ -6294,7 +6294,7 @@
         <v>56</v>
       </c>
       <c r="I22" s="16">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>57</v>
@@ -6326,7 +6326,7 @@
         <v>56</v>
       </c>
       <c r="I23" s="18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J23" s="18" t="s">
         <v>57</v>
@@ -6358,7 +6358,7 @@
         <v>56</v>
       </c>
       <c r="I24" s="16">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J24" s="16" t="s">
         <v>57</v>
@@ -6390,7 +6390,7 @@
         <v>56</v>
       </c>
       <c r="I25" s="18">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J25" s="18" t="s">
         <v>57</v>
@@ -6422,7 +6422,7 @@
         <v>56</v>
       </c>
       <c r="I26" s="16">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J26" s="16" t="s">
         <v>57</v>
@@ -6454,7 +6454,7 @@
         <v>56</v>
       </c>
       <c r="I27" s="18">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J27" s="18" t="s">
         <v>57</v>
@@ -6486,7 +6486,7 @@
         <v>56</v>
       </c>
       <c r="I28" s="16">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J28" s="16" t="s">
         <v>57</v>
@@ -6518,7 +6518,7 @@
         <v>56</v>
       </c>
       <c r="I29" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J29" s="18" t="s">
         <v>57</v>
@@ -6550,7 +6550,7 @@
         <v>56</v>
       </c>
       <c r="I30" s="16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J30" s="16" t="s">
         <v>57</v>
@@ -6582,7 +6582,7 @@
         <v>56</v>
       </c>
       <c r="I31" s="18">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J31" s="18" t="s">
         <v>57</v>
@@ -6614,7 +6614,7 @@
         <v>56</v>
       </c>
       <c r="I32" s="16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>57</v>
@@ -6646,7 +6646,7 @@
         <v>56</v>
       </c>
       <c r="I33" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J33" s="18" t="s">
         <v>57</v>
@@ -6710,7 +6710,7 @@
         <v>56</v>
       </c>
       <c r="I35" s="18">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J35" s="18" t="s">
         <v>57</v>
@@ -6742,7 +6742,7 @@
         <v>56</v>
       </c>
       <c r="I36" s="16">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J36" s="16" t="s">
         <v>57</v>
@@ -6774,7 +6774,7 @@
         <v>56</v>
       </c>
       <c r="I37" s="18">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J37" s="18" t="s">
         <v>57</v>
@@ -6806,7 +6806,7 @@
         <v>56</v>
       </c>
       <c r="I38" s="16">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J38" s="16" t="s">
         <v>57</v>
@@ -6838,7 +6838,7 @@
         <v>56</v>
       </c>
       <c r="I39" s="18">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J39" s="18" t="s">
         <v>57</v>
@@ -6902,7 +6902,7 @@
         <v>56</v>
       </c>
       <c r="I41" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J41" s="18" t="s">
         <v>57</v>
@@ -6934,7 +6934,7 @@
         <v>56</v>
       </c>
       <c r="I42" s="16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J42" s="16" t="s">
         <v>57</v>
@@ -6966,7 +6966,7 @@
         <v>56</v>
       </c>
       <c r="I43" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J43" s="18" t="s">
         <v>57</v>
@@ -6998,7 +6998,7 @@
         <v>56</v>
       </c>
       <c r="I44" s="16">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J44" s="16" t="s">
         <v>57</v>
@@ -7030,7 +7030,7 @@
         <v>56</v>
       </c>
       <c r="I45" s="18">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J45" s="18" t="s">
         <v>57</v>
@@ -7094,7 +7094,7 @@
         <v>56</v>
       </c>
       <c r="I47" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J47" s="18" t="s">
         <v>57</v>
@@ -7126,7 +7126,7 @@
         <v>56</v>
       </c>
       <c r="I48" s="16">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J48" s="16" t="s">
         <v>57</v>
@@ -7158,7 +7158,7 @@
         <v>56</v>
       </c>
       <c r="I49" s="18">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J49" s="18" t="s">
         <v>57</v>
@@ -7190,7 +7190,7 @@
         <v>56</v>
       </c>
       <c r="I50" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J50" s="16" t="s">
         <v>57</v>
@@ -7222,7 +7222,7 @@
         <v>56</v>
       </c>
       <c r="I51" s="18">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J51" s="18" t="s">
         <v>57</v>
@@ -7254,7 +7254,7 @@
         <v>56</v>
       </c>
       <c r="I52" s="16">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J52" s="16" t="s">
         <v>57</v>
@@ -7286,7 +7286,7 @@
         <v>56</v>
       </c>
       <c r="I53" s="18">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J53" s="18" t="s">
         <v>57</v>
@@ -7350,7 +7350,7 @@
         <v>56</v>
       </c>
       <c r="I55" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J55" s="18" t="s">
         <v>57</v>
@@ -7382,7 +7382,7 @@
         <v>56</v>
       </c>
       <c r="I56" s="16">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J56" s="16" t="s">
         <v>57</v>
@@ -7414,7 +7414,7 @@
         <v>56</v>
       </c>
       <c r="I57" s="18">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J57" s="18" t="s">
         <v>57</v>
@@ -7478,7 +7478,7 @@
         <v>56</v>
       </c>
       <c r="I59" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J59" s="18" t="s">
         <v>57</v>
@@ -7510,7 +7510,7 @@
         <v>56</v>
       </c>
       <c r="I60" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J60" s="16" t="s">
         <v>57</v>
@@ -7542,7 +7542,7 @@
         <v>56</v>
       </c>
       <c r="I61" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J61" s="18" t="s">
         <v>57</v>
@@ -7574,7 +7574,7 @@
         <v>56</v>
       </c>
       <c r="I62" s="16">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J62" s="16" t="s">
         <v>57</v>
@@ -7606,7 +7606,7 @@
         <v>56</v>
       </c>
       <c r="I63" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J63" s="18" t="s">
         <v>57</v>
@@ -7638,7 +7638,7 @@
         <v>56</v>
       </c>
       <c r="I64" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J64" s="16" t="s">
         <v>57</v>
@@ -7670,7 +7670,7 @@
         <v>56</v>
       </c>
       <c r="I65" s="18">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J65" s="18" t="s">
         <v>57</v>
@@ -7702,7 +7702,7 @@
         <v>56</v>
       </c>
       <c r="I66" s="16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J66" s="16" t="s">
         <v>57</v>
@@ -7734,7 +7734,7 @@
         <v>56</v>
       </c>
       <c r="I67" s="18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J67" s="18" t="s">
         <v>57</v>
@@ -7766,7 +7766,7 @@
         <v>56</v>
       </c>
       <c r="I68" s="16">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J68" s="16" t="s">
         <v>57</v>
@@ -7798,7 +7798,7 @@
         <v>56</v>
       </c>
       <c r="I69" s="18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J69" s="18" t="s">
         <v>57</v>
@@ -7830,7 +7830,7 @@
         <v>56</v>
       </c>
       <c r="I70" s="16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J70" s="16" t="s">
         <v>57</v>
@@ -7862,7 +7862,7 @@
         <v>56</v>
       </c>
       <c r="I71" s="18">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J71" s="18" t="s">
         <v>57</v>
@@ -7926,7 +7926,7 @@
         <v>56</v>
       </c>
       <c r="I73" s="18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J73" s="18" t="s">
         <v>57</v>
@@ -7958,7 +7958,7 @@
         <v>56</v>
       </c>
       <c r="I74" s="16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J74" s="16" t="s">
         <v>57</v>
@@ -7990,7 +7990,7 @@
         <v>56</v>
       </c>
       <c r="I75" s="18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J75" s="18" t="s">
         <v>57</v>
@@ -8022,7 +8022,7 @@
         <v>56</v>
       </c>
       <c r="I76" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="16" t="s">
         <v>57</v>
@@ -8054,7 +8054,7 @@
         <v>56</v>
       </c>
       <c r="I77" s="18">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J77" s="18" t="s">
         <v>57</v>
@@ -8086,7 +8086,7 @@
         <v>56</v>
       </c>
       <c r="I78" s="16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J78" s="16" t="s">
         <v>57</v>
@@ -8118,7 +8118,7 @@
         <v>56</v>
       </c>
       <c r="I79" s="18">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J79" s="18" t="s">
         <v>57</v>
@@ -8182,7 +8182,7 @@
         <v>56</v>
       </c>
       <c r="I81" s="18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J81" s="18" t="s">
         <v>57</v>
@@ -8214,7 +8214,7 @@
         <v>56</v>
       </c>
       <c r="I82" s="16">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J82" s="16" t="s">
         <v>57</v>
@@ -8246,7 +8246,7 @@
         <v>56</v>
       </c>
       <c r="I83" s="18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J83" s="18" t="s">
         <v>57</v>
@@ -8278,7 +8278,7 @@
         <v>56</v>
       </c>
       <c r="I84" s="16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J84" s="16" t="s">
         <v>57</v>
@@ -8310,7 +8310,7 @@
         <v>56</v>
       </c>
       <c r="I85" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J85" s="18" t="s">
         <v>57</v>
@@ -8342,7 +8342,7 @@
         <v>56</v>
       </c>
       <c r="I86" s="16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J86" s="16" t="s">
         <v>57</v>
@@ -8374,7 +8374,7 @@
         <v>56</v>
       </c>
       <c r="I87" s="18">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J87" s="18" t="s">
         <v>57</v>
@@ -8406,7 +8406,7 @@
         <v>56</v>
       </c>
       <c r="I88" s="16">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J88" s="16" t="s">
         <v>57</v>
@@ -8438,7 +8438,7 @@
         <v>56</v>
       </c>
       <c r="I89" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J89" s="18" t="s">
         <v>57</v>
@@ -8470,7 +8470,7 @@
         <v>56</v>
       </c>
       <c r="I90" s="16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J90" s="16" t="s">
         <v>57</v>
@@ -8502,7 +8502,7 @@
         <v>56</v>
       </c>
       <c r="I91" s="18">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J91" s="18" t="s">
         <v>57</v>
@@ -8534,7 +8534,7 @@
         <v>56</v>
       </c>
       <c r="I92" s="16">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J92" s="16" t="s">
         <v>57</v>
@@ -8566,7 +8566,7 @@
         <v>56</v>
       </c>
       <c r="I93" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J93" s="18" t="s">
         <v>57</v>
@@ -8598,7 +8598,7 @@
         <v>56</v>
       </c>
       <c r="I94" s="16">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J94" s="16" t="s">
         <v>57</v>
@@ -8630,7 +8630,7 @@
         <v>56</v>
       </c>
       <c r="I95" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J95" s="18" t="s">
         <v>57</v>
@@ -8662,7 +8662,7 @@
         <v>56</v>
       </c>
       <c r="I96" s="16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J96" s="16" t="s">
         <v>57</v>
@@ -8694,7 +8694,7 @@
         <v>56</v>
       </c>
       <c r="I97" s="18">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J97" s="18" t="s">
         <v>57</v>
@@ -8726,7 +8726,7 @@
         <v>56</v>
       </c>
       <c r="I98" s="16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J98" s="16" t="s">
         <v>57</v>
@@ -8758,7 +8758,7 @@
         <v>56</v>
       </c>
       <c r="I99" s="18">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J99" s="18" t="s">
         <v>57</v>
@@ -8790,7 +8790,7 @@
         <v>56</v>
       </c>
       <c r="I100" s="16">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J100" s="16" t="s">
         <v>57</v>
@@ -8822,7 +8822,7 @@
         <v>56</v>
       </c>
       <c r="I101" s="18">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J101" s="18" t="s">
         <v>57</v>
@@ -8854,7 +8854,7 @@
         <v>56</v>
       </c>
       <c r="I102" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J102" s="16" t="s">
         <v>57</v>
@@ -8886,7 +8886,7 @@
         <v>56</v>
       </c>
       <c r="I103" s="18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J103" s="18" t="s">
         <v>57</v>
@@ -8918,7 +8918,7 @@
         <v>56</v>
       </c>
       <c r="I104" s="16">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J104" s="16" t="s">
         <v>57</v>
@@ -8950,7 +8950,7 @@
         <v>56</v>
       </c>
       <c r="I105" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J105" s="18" t="s">
         <v>57</v>
@@ -8982,7 +8982,7 @@
         <v>56</v>
       </c>
       <c r="I106" s="16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J106" s="16" t="s">
         <v>57</v>
@@ -9014,7 +9014,7 @@
         <v>56</v>
       </c>
       <c r="I107" s="18">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J107" s="18" t="s">
         <v>57</v>
@@ -9046,7 +9046,7 @@
         <v>56</v>
       </c>
       <c r="I108" s="16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J108" s="16" t="s">
         <v>57</v>
@@ -9078,7 +9078,7 @@
         <v>56</v>
       </c>
       <c r="I109" s="18">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J109" s="18" t="s">
         <v>57</v>
@@ -9142,7 +9142,7 @@
         <v>56</v>
       </c>
       <c r="I111" s="18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J111" s="18" t="s">
         <v>57</v>
@@ -9174,7 +9174,7 @@
         <v>56</v>
       </c>
       <c r="I112" s="16">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J112" s="16" t="s">
         <v>57</v>
@@ -9206,7 +9206,7 @@
         <v>56</v>
       </c>
       <c r="I113" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J113" s="18" t="s">
         <v>57</v>
@@ -9238,7 +9238,7 @@
         <v>56</v>
       </c>
       <c r="I114" s="16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J114" s="16" t="s">
         <v>57</v>
@@ -9270,7 +9270,7 @@
         <v>56</v>
       </c>
       <c r="I115" s="18">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J115" s="18" t="s">
         <v>57</v>
@@ -9302,7 +9302,7 @@
         <v>56</v>
       </c>
       <c r="I116" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J116" s="16" t="s">
         <v>57</v>
@@ -9334,7 +9334,7 @@
         <v>56</v>
       </c>
       <c r="I117" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J117" s="18" t="s">
         <v>57</v>
@@ -9366,7 +9366,7 @@
         <v>56</v>
       </c>
       <c r="I118" s="16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J118" s="16" t="s">
         <v>57</v>
@@ -9398,7 +9398,7 @@
         <v>56</v>
       </c>
       <c r="I119" s="18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J119" s="18" t="s">
         <v>57</v>
@@ -9430,7 +9430,7 @@
         <v>56</v>
       </c>
       <c r="I120" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J120" s="16" t="s">
         <v>57</v>
@@ -9526,7 +9526,7 @@
         <v>56</v>
       </c>
       <c r="I123" s="18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J123" s="18" t="s">
         <v>57</v>
@@ -9558,7 +9558,7 @@
         <v>56</v>
       </c>
       <c r="I124" s="16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J124" s="16" t="s">
         <v>57</v>
@@ -9590,7 +9590,7 @@
         <v>56</v>
       </c>
       <c r="I125" s="18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J125" s="18" t="s">
         <v>57</v>
@@ -9622,7 +9622,7 @@
         <v>56</v>
       </c>
       <c r="I126" s="16">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J126" s="16" t="s">
         <v>57</v>
@@ -9654,7 +9654,7 @@
         <v>56</v>
       </c>
       <c r="I127" s="18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J127" s="18" t="s">
         <v>57</v>
@@ -9686,7 +9686,7 @@
         <v>56</v>
       </c>
       <c r="I128" s="16">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J128" s="16" t="s">
         <v>57</v>
@@ -9718,7 +9718,7 @@
         <v>56</v>
       </c>
       <c r="I129" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J129" s="18" t="s">
         <v>57</v>
@@ -9750,7 +9750,7 @@
         <v>56</v>
       </c>
       <c r="I130" s="16">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J130" s="16" t="s">
         <v>57</v>
@@ -9782,7 +9782,7 @@
         <v>56</v>
       </c>
       <c r="I131" s="18">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J131" s="18" t="s">
         <v>57</v>
@@ -9814,7 +9814,7 @@
         <v>56</v>
       </c>
       <c r="I132" s="16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J132" s="16" t="s">
         <v>57</v>
@@ -9846,7 +9846,7 @@
         <v>56</v>
       </c>
       <c r="I133" s="18">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J133" s="18" t="s">
         <v>57</v>
@@ -9878,7 +9878,7 @@
         <v>56</v>
       </c>
       <c r="I134" s="16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J134" s="16" t="s">
         <v>57</v>
@@ -9910,7 +9910,7 @@
         <v>56</v>
       </c>
       <c r="I135" s="18">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J135" s="18" t="s">
         <v>57</v>
@@ -9942,7 +9942,7 @@
         <v>56</v>
       </c>
       <c r="I136" s="16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J136" s="16" t="s">
         <v>57</v>
@@ -9974,7 +9974,7 @@
         <v>56</v>
       </c>
       <c r="I137" s="18">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J137" s="18" t="s">
         <v>57</v>
@@ -10006,7 +10006,7 @@
         <v>56</v>
       </c>
       <c r="I138" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J138" s="16" t="s">
         <v>57</v>
@@ -10038,7 +10038,7 @@
         <v>56</v>
       </c>
       <c r="I139" s="18">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J139" s="18" t="s">
         <v>57</v>
@@ -10070,7 +10070,7 @@
         <v>56</v>
       </c>
       <c r="I140" s="16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J140" s="16" t="s">
         <v>57</v>
@@ -10102,7 +10102,7 @@
         <v>56</v>
       </c>
       <c r="I141" s="18">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J141" s="18" t="s">
         <v>57</v>
@@ -10134,7 +10134,7 @@
         <v>56</v>
       </c>
       <c r="I142" s="16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J142" s="16" t="s">
         <v>57</v>
@@ -10166,7 +10166,7 @@
         <v>56</v>
       </c>
       <c r="I143" s="18">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J143" s="18" t="s">
         <v>57</v>
@@ -10230,7 +10230,7 @@
         <v>56</v>
       </c>
       <c r="I145" s="18">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J145" s="18" t="s">
         <v>57</v>
@@ -10294,7 +10294,7 @@
         <v>56</v>
       </c>
       <c r="I147" s="18">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J147" s="18" t="s">
         <v>57</v>
@@ -10326,7 +10326,7 @@
         <v>56</v>
       </c>
       <c r="I148" s="16">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J148" s="16" t="s">
         <v>57</v>
@@ -10358,7 +10358,7 @@
         <v>56</v>
       </c>
       <c r="I149" s="18">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J149" s="18" t="s">
         <v>57</v>
@@ -10390,7 +10390,7 @@
         <v>56</v>
       </c>
       <c r="I150" s="16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J150" s="16" t="s">
         <v>57</v>
@@ -10422,7 +10422,7 @@
         <v>56</v>
       </c>
       <c r="I151" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J151" s="18" t="s">
         <v>57</v>
@@ -10486,7 +10486,7 @@
         <v>56</v>
       </c>
       <c r="I153" s="18">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J153" s="18" t="s">
         <v>57</v>
@@ -10518,7 +10518,7 @@
         <v>56</v>
       </c>
       <c r="I154" s="16">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J154" s="16" t="s">
         <v>57</v>
@@ -10550,7 +10550,7 @@
         <v>56</v>
       </c>
       <c r="I155" s="18">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J155" s="18" t="s">
         <v>57</v>
@@ -10582,7 +10582,7 @@
         <v>56</v>
       </c>
       <c r="I156" s="16">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J156" s="16" t="s">
         <v>57</v>
@@ -10614,7 +10614,7 @@
         <v>56</v>
       </c>
       <c r="I157" s="18">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J157" s="18" t="s">
         <v>57</v>
@@ -10646,7 +10646,7 @@
         <v>56</v>
       </c>
       <c r="I158" s="16">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J158" s="16" t="s">
         <v>57</v>
@@ -10678,7 +10678,7 @@
         <v>56</v>
       </c>
       <c r="I159" s="18">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J159" s="18" t="s">
         <v>57</v>
@@ -10710,7 +10710,7 @@
         <v>56</v>
       </c>
       <c r="I160" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J160" s="16" t="s">
         <v>57</v>
@@ -10742,7 +10742,7 @@
         <v>56</v>
       </c>
       <c r="I161" s="18">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J161" s="18" t="s">
         <v>57</v>
@@ -10774,7 +10774,7 @@
         <v>56</v>
       </c>
       <c r="I162" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J162" s="16" t="s">
         <v>57</v>
@@ -10838,7 +10838,7 @@
         <v>56</v>
       </c>
       <c r="I164" s="16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J164" s="16" t="s">
         <v>57</v>
@@ -10870,7 +10870,7 @@
         <v>56</v>
       </c>
       <c r="I165" s="18">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J165" s="18" t="s">
         <v>57</v>
@@ -10902,7 +10902,7 @@
         <v>56</v>
       </c>
       <c r="I166" s="16">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J166" s="16" t="s">
         <v>57</v>
@@ -10934,7 +10934,7 @@
         <v>56</v>
       </c>
       <c r="I167" s="18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J167" s="18" t="s">
         <v>57</v>
@@ -10966,7 +10966,7 @@
         <v>56</v>
       </c>
       <c r="I168" s="16">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J168" s="16" t="s">
         <v>57</v>
@@ -10998,7 +10998,7 @@
         <v>56</v>
       </c>
       <c r="I169" s="18">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J169" s="18" t="s">
         <v>57</v>
@@ -11030,7 +11030,7 @@
         <v>56</v>
       </c>
       <c r="I170" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J170" s="16" t="s">
         <v>57</v>
@@ -11062,7 +11062,7 @@
         <v>56</v>
       </c>
       <c r="I171" s="18">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J171" s="18" t="s">
         <v>57</v>
@@ -11094,7 +11094,7 @@
         <v>56</v>
       </c>
       <c r="I172" s="16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J172" s="16" t="s">
         <v>57</v>
@@ -11126,7 +11126,7 @@
         <v>56</v>
       </c>
       <c r="I173" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J173" s="18" t="s">
         <v>57</v>
@@ -11158,7 +11158,7 @@
         <v>56</v>
       </c>
       <c r="I174" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J174" s="16" t="s">
         <v>57</v>
@@ -11222,7 +11222,7 @@
         <v>56</v>
       </c>
       <c r="I176" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J176" s="16" t="s">
         <v>57</v>
@@ -11254,7 +11254,7 @@
         <v>56</v>
       </c>
       <c r="I177" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J177" s="18" t="s">
         <v>57</v>
@@ -11286,7 +11286,7 @@
         <v>56</v>
       </c>
       <c r="I178" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J178" s="16" t="s">
         <v>57</v>
@@ -11318,7 +11318,7 @@
         <v>56</v>
       </c>
       <c r="I179" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J179" s="18" t="s">
         <v>57</v>
@@ -11350,7 +11350,7 @@
         <v>56</v>
       </c>
       <c r="I180" s="16">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J180" s="16" t="s">
         <v>57</v>
@@ -11382,7 +11382,7 @@
         <v>56</v>
       </c>
       <c r="I181" s="18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J181" s="18" t="s">
         <v>57</v>
@@ -11414,7 +11414,7 @@
         <v>56</v>
       </c>
       <c r="I182" s="16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J182" s="16" t="s">
         <v>57</v>
@@ -11446,7 +11446,7 @@
         <v>56</v>
       </c>
       <c r="I183" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J183" s="18" t="s">
         <v>57</v>
@@ -11478,7 +11478,7 @@
         <v>56</v>
       </c>
       <c r="I184" s="16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J184" s="16" t="s">
         <v>57</v>
@@ -11542,7 +11542,7 @@
         <v>56</v>
       </c>
       <c r="I186" s="16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J186" s="16" t="s">
         <v>57</v>
@@ -11606,7 +11606,7 @@
         <v>56</v>
       </c>
       <c r="I188" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J188" s="16" t="s">
         <v>57</v>
@@ -11638,7 +11638,7 @@
         <v>56</v>
       </c>
       <c r="I189" s="18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J189" s="18" t="s">
         <v>57</v>
@@ -11670,7 +11670,7 @@
         <v>56</v>
       </c>
       <c r="I190" s="16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J190" s="16" t="s">
         <v>57</v>
@@ -11702,7 +11702,7 @@
         <v>56</v>
       </c>
       <c r="I191" s="18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J191" s="18" t="s">
         <v>57</v>
@@ -11734,7 +11734,7 @@
         <v>56</v>
       </c>
       <c r="I192" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J192" s="16" t="s">
         <v>57</v>
@@ -11766,7 +11766,7 @@
         <v>56</v>
       </c>
       <c r="I193" s="18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J193" s="18" t="s">
         <v>57</v>
@@ -11798,7 +11798,7 @@
         <v>56</v>
       </c>
       <c r="I194" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J194" s="16" t="s">
         <v>57</v>
@@ -11830,7 +11830,7 @@
         <v>56</v>
       </c>
       <c r="I195" s="18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J195" s="18" t="s">
         <v>57</v>
@@ -11862,7 +11862,7 @@
         <v>56</v>
       </c>
       <c r="I196" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J196" s="16" t="s">
         <v>57</v>
@@ -11894,7 +11894,7 @@
         <v>56</v>
       </c>
       <c r="I197" s="18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J197" s="18" t="s">
         <v>57</v>
@@ -11926,7 +11926,7 @@
         <v>56</v>
       </c>
       <c r="I198" s="16">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J198" s="16" t="s">
         <v>57</v>
@@ -11958,7 +11958,7 @@
         <v>56</v>
       </c>
       <c r="I199" s="18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J199" s="18" t="s">
         <v>57</v>
@@ -11990,7 +11990,7 @@
         <v>56</v>
       </c>
       <c r="I200" s="16">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J200" s="16" t="s">
         <v>57</v>
@@ -12022,7 +12022,7 @@
         <v>56</v>
       </c>
       <c r="I201" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J201" s="18" t="s">
         <v>57</v>
@@ -12054,7 +12054,7 @@
         <v>56</v>
       </c>
       <c r="I202" s="16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J202" s="16" t="s">
         <v>57</v>
@@ -12086,7 +12086,7 @@
         <v>56</v>
       </c>
       <c r="I203" s="18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J203" s="18" t="s">
         <v>57</v>
@@ -12118,7 +12118,7 @@
         <v>56</v>
       </c>
       <c r="I204" s="16">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J204" s="16" t="s">
         <v>57</v>
@@ -12150,7 +12150,7 @@
         <v>56</v>
       </c>
       <c r="I205" s="18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J205" s="18" t="s">
         <v>57</v>
@@ -12182,7 +12182,7 @@
         <v>56</v>
       </c>
       <c r="I206" s="16">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J206" s="16" t="s">
         <v>57</v>
@@ -12214,7 +12214,7 @@
         <v>56</v>
       </c>
       <c r="I207" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J207" s="18" t="s">
         <v>57</v>
@@ -12246,7 +12246,7 @@
         <v>56</v>
       </c>
       <c r="I208" s="16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J208" s="16" t="s">
         <v>57</v>
@@ -12278,7 +12278,7 @@
         <v>56</v>
       </c>
       <c r="I209" s="18">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J209" s="18" t="s">
         <v>57</v>
@@ -12342,7 +12342,7 @@
         <v>56</v>
       </c>
       <c r="I211" s="18">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J211" s="18" t="s">
         <v>57</v>
@@ -12374,7 +12374,7 @@
         <v>56</v>
       </c>
       <c r="I212" s="16">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J212" s="16" t="s">
         <v>57</v>
@@ -12406,7 +12406,7 @@
         <v>56</v>
       </c>
       <c r="I213" s="18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J213" s="18" t="s">
         <v>57</v>
@@ -12470,7 +12470,7 @@
         <v>56</v>
       </c>
       <c r="I215" s="18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J215" s="18" t="s">
         <v>57</v>
@@ -12502,7 +12502,7 @@
         <v>56</v>
       </c>
       <c r="I216" s="16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J216" s="16" t="s">
         <v>57</v>
@@ -12566,7 +12566,7 @@
         <v>56</v>
       </c>
       <c r="I218" s="16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J218" s="16" t="s">
         <v>57</v>
@@ -12598,7 +12598,7 @@
         <v>56</v>
       </c>
       <c r="I219" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J219" s="18" t="s">
         <v>57</v>
@@ -12630,7 +12630,7 @@
         <v>56</v>
       </c>
       <c r="I220" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J220" s="16" t="s">
         <v>57</v>
@@ -12662,7 +12662,7 @@
         <v>56</v>
       </c>
       <c r="I221" s="18">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J221" s="18" t="s">
         <v>57</v>
@@ -12726,7 +12726,7 @@
         <v>56</v>
       </c>
       <c r="I223" s="18">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J223" s="18" t="s">
         <v>57</v>
@@ -12758,7 +12758,7 @@
         <v>56</v>
       </c>
       <c r="I224" s="16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J224" s="16" t="s">
         <v>57</v>
@@ -12790,7 +12790,7 @@
         <v>56</v>
       </c>
       <c r="I225" s="18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J225" s="18" t="s">
         <v>57</v>
@@ -12822,7 +12822,7 @@
         <v>56</v>
       </c>
       <c r="I226" s="16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J226" s="16" t="s">
         <v>57</v>
@@ -12854,7 +12854,7 @@
         <v>56</v>
       </c>
       <c r="I227" s="18">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J227" s="18" t="s">
         <v>57</v>
@@ -12886,7 +12886,7 @@
         <v>56</v>
       </c>
       <c r="I228" s="16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J228" s="16" t="s">
         <v>57</v>
@@ -12918,7 +12918,7 @@
         <v>56</v>
       </c>
       <c r="I229" s="18">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J229" s="18" t="s">
         <v>57</v>
@@ -12950,7 +12950,7 @@
         <v>56</v>
       </c>
       <c r="I230" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J230" s="16" t="s">
         <v>57</v>
@@ -12982,7 +12982,7 @@
         <v>56</v>
       </c>
       <c r="I231" s="18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J231" s="18" t="s">
         <v>57</v>
@@ -13014,7 +13014,7 @@
         <v>56</v>
       </c>
       <c r="I232" s="16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J232" s="16" t="s">
         <v>57</v>
@@ -13046,7 +13046,7 @@
         <v>56</v>
       </c>
       <c r="I233" s="18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J233" s="18" t="s">
         <v>57</v>
@@ -13078,7 +13078,7 @@
         <v>56</v>
       </c>
       <c r="I234" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J234" s="16" t="s">
         <v>57</v>
@@ -13110,7 +13110,7 @@
         <v>56</v>
       </c>
       <c r="I235" s="18">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J235" s="18" t="s">
         <v>57</v>
@@ -13142,7 +13142,7 @@
         <v>56</v>
       </c>
       <c r="I236" s="16">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J236" s="16" t="s">
         <v>57</v>
@@ -13206,7 +13206,7 @@
         <v>56</v>
       </c>
       <c r="I238" s="16">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J238" s="16" t="s">
         <v>57</v>
@@ -13238,7 +13238,7 @@
         <v>56</v>
       </c>
       <c r="I239" s="18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J239" s="18" t="s">
         <v>57</v>
@@ -13270,7 +13270,7 @@
         <v>56</v>
       </c>
       <c r="I240" s="16">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J240" s="16" t="s">
         <v>57</v>
@@ -13302,7 +13302,7 @@
         <v>56</v>
       </c>
       <c r="I241" s="18">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J241" s="18" t="s">
         <v>57</v>
@@ -13334,7 +13334,7 @@
         <v>56</v>
       </c>
       <c r="I242" s="16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J242" s="16" t="s">
         <v>57</v>
@@ -13366,7 +13366,7 @@
         <v>56</v>
       </c>
       <c r="I243" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J243" s="18" t="s">
         <v>57</v>
@@ -13398,7 +13398,7 @@
         <v>56</v>
       </c>
       <c r="I244" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J244" s="16" t="s">
         <v>57</v>
@@ -13462,7 +13462,7 @@
         <v>56</v>
       </c>
       <c r="I246" s="16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J246" s="16" t="s">
         <v>57</v>
@@ -13494,7 +13494,7 @@
         <v>56</v>
       </c>
       <c r="I247" s="18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J247" s="18" t="s">
         <v>57</v>
@@ -13526,7 +13526,7 @@
         <v>56</v>
       </c>
       <c r="I248" s="16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J248" s="16" t="s">
         <v>57</v>
@@ -13558,7 +13558,7 @@
         <v>56</v>
       </c>
       <c r="I249" s="18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J249" s="18" t="s">
         <v>57</v>
@@ -13590,7 +13590,7 @@
         <v>56</v>
       </c>
       <c r="I250" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J250" s="16" t="s">
         <v>57</v>
@@ -13622,7 +13622,7 @@
         <v>56</v>
       </c>
       <c r="I251" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J251" s="18" t="s">
         <v>57</v>
@@ -13654,7 +13654,7 @@
         <v>56</v>
       </c>
       <c r="I252" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J252" s="16" t="s">
         <v>57</v>
@@ -13718,7 +13718,7 @@
         <v>56</v>
       </c>
       <c r="I254" s="16">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J254" s="16" t="s">
         <v>57</v>
@@ -13782,7 +13782,7 @@
         <v>56</v>
       </c>
       <c r="I256" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J256" s="16" t="s">
         <v>57</v>
@@ -13814,7 +13814,7 @@
         <v>56</v>
       </c>
       <c r="I257" s="18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J257" s="18" t="s">
         <v>57</v>
@@ -13846,7 +13846,7 @@
         <v>56</v>
       </c>
       <c r="I258" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J258" s="16" t="s">
         <v>57</v>
@@ -13878,7 +13878,7 @@
         <v>56</v>
       </c>
       <c r="I259" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J259" s="18" t="s">
         <v>57</v>
@@ -13910,7 +13910,7 @@
         <v>56</v>
       </c>
       <c r="I260" s="16">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J260" s="16" t="s">
         <v>57</v>
@@ -13942,7 +13942,7 @@
         <v>56</v>
       </c>
       <c r="I261" s="18">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J261" s="18" t="s">
         <v>57</v>
@@ -13974,7 +13974,7 @@
         <v>56</v>
       </c>
       <c r="I262" s="16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J262" s="16" t="s">
         <v>57</v>
@@ -14006,7 +14006,7 @@
         <v>56</v>
       </c>
       <c r="I263" s="18">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J263" s="18" t="s">
         <v>57</v>
@@ -14038,7 +14038,7 @@
         <v>56</v>
       </c>
       <c r="I264" s="16">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J264" s="16" t="s">
         <v>57</v>
@@ -14070,7 +14070,7 @@
         <v>56</v>
       </c>
       <c r="I265" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J265" s="18" t="s">
         <v>57</v>
@@ -14102,7 +14102,7 @@
         <v>56</v>
       </c>
       <c r="I266" s="16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J266" s="16" t="s">
         <v>57</v>
@@ -14134,7 +14134,7 @@
         <v>56</v>
       </c>
       <c r="I267" s="18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J267" s="18" t="s">
         <v>57</v>
@@ -14166,7 +14166,7 @@
         <v>56</v>
       </c>
       <c r="I268" s="16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J268" s="16" t="s">
         <v>57</v>
@@ -14198,7 +14198,7 @@
         <v>56</v>
       </c>
       <c r="I269" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J269" s="18" t="s">
         <v>57</v>
@@ -14262,7 +14262,7 @@
         <v>56</v>
       </c>
       <c r="I271" s="18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J271" s="18" t="s">
         <v>57</v>
@@ -14294,7 +14294,7 @@
         <v>56</v>
       </c>
       <c r="I272" s="16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J272" s="16" t="s">
         <v>57</v>
@@ -14326,7 +14326,7 @@
         <v>56</v>
       </c>
       <c r="I273" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J273" s="18" t="s">
         <v>57</v>
@@ -14358,7 +14358,7 @@
         <v>56</v>
       </c>
       <c r="I274" s="16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J274" s="16" t="s">
         <v>57</v>
@@ -14390,7 +14390,7 @@
         <v>56</v>
       </c>
       <c r="I275" s="18">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J275" s="18" t="s">
         <v>57</v>
@@ -14422,7 +14422,7 @@
         <v>56</v>
       </c>
       <c r="I276" s="16">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J276" s="16" t="s">
         <v>57</v>
@@ -14454,7 +14454,7 @@
         <v>56</v>
       </c>
       <c r="I277" s="18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J277" s="18" t="s">
         <v>57</v>
@@ -14486,7 +14486,7 @@
         <v>56</v>
       </c>
       <c r="I278" s="16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J278" s="16" t="s">
         <v>57</v>
@@ -14518,7 +14518,7 @@
         <v>56</v>
       </c>
       <c r="I279" s="18">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J279" s="18" t="s">
         <v>57</v>
@@ -14550,7 +14550,7 @@
         <v>56</v>
       </c>
       <c r="I280" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J280" s="16" t="s">
         <v>57</v>
@@ -14582,7 +14582,7 @@
         <v>56</v>
       </c>
       <c r="I281" s="18">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J281" s="18" t="s">
         <v>57</v>
@@ -14614,7 +14614,7 @@
         <v>56</v>
       </c>
       <c r="I282" s="16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J282" s="16" t="s">
         <v>57</v>
@@ -14646,7 +14646,7 @@
         <v>56</v>
       </c>
       <c r="I283" s="18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J283" s="18" t="s">
         <v>57</v>
@@ -14710,7 +14710,7 @@
         <v>56</v>
       </c>
       <c r="I285" s="18">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J285" s="18" t="s">
         <v>57</v>
@@ -14742,7 +14742,7 @@
         <v>56</v>
       </c>
       <c r="I286" s="16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J286" s="16" t="s">
         <v>57</v>
@@ -14774,7 +14774,7 @@
         <v>56</v>
       </c>
       <c r="I287" s="18">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J287" s="18" t="s">
         <v>57</v>
@@ -14806,7 +14806,7 @@
         <v>56</v>
       </c>
       <c r="I288" s="16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J288" s="16" t="s">
         <v>57</v>
@@ -14870,7 +14870,7 @@
         <v>56</v>
       </c>
       <c r="I290" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J290" s="16" t="s">
         <v>57</v>
@@ -14902,7 +14902,7 @@
         <v>56</v>
       </c>
       <c r="I291" s="18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J291" s="18" t="s">
         <v>57</v>
@@ -14934,7 +14934,7 @@
         <v>56</v>
       </c>
       <c r="I292" s="16">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J292" s="16" t="s">
         <v>57</v>
@@ -14998,7 +14998,7 @@
         <v>56</v>
       </c>
       <c r="I294" s="16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J294" s="16" t="s">
         <v>57</v>
@@ -15094,7 +15094,7 @@
         <v>56</v>
       </c>
       <c r="I297" s="18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J297" s="18" t="s">
         <v>57</v>
@@ -15126,7 +15126,7 @@
         <v>56</v>
       </c>
       <c r="I298" s="16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J298" s="16" t="s">
         <v>57</v>
@@ -15158,7 +15158,7 @@
         <v>56</v>
       </c>
       <c r="I299" s="18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J299" s="18" t="s">
         <v>57</v>
@@ -15190,7 +15190,7 @@
         <v>56</v>
       </c>
       <c r="I300" s="16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J300" s="16" t="s">
         <v>57</v>
@@ -15222,7 +15222,7 @@
         <v>56</v>
       </c>
       <c r="I301" s="18">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J301" s="18" t="s">
         <v>57</v>
@@ -15254,7 +15254,7 @@
         <v>56</v>
       </c>
       <c r="I302" s="16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J302" s="16" t="s">
         <v>57</v>
@@ -15318,7 +15318,7 @@
         <v>56</v>
       </c>
       <c r="I304" s="16">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J304" s="16" t="s">
         <v>57</v>
@@ -15350,7 +15350,7 @@
         <v>56</v>
       </c>
       <c r="I305" s="18">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J305" s="18" t="s">
         <v>57</v>
@@ -15414,7 +15414,7 @@
         <v>56</v>
       </c>
       <c r="I307" s="18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J307" s="18" t="s">
         <v>57</v>
@@ -15446,7 +15446,7 @@
         <v>56</v>
       </c>
       <c r="I308" s="16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J308" s="16" t="s">
         <v>57</v>
@@ -15478,7 +15478,7 @@
         <v>56</v>
       </c>
       <c r="I309" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J309" s="18" t="s">
         <v>57</v>
@@ -15510,7 +15510,7 @@
         <v>56</v>
       </c>
       <c r="I310" s="16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J310" s="16" t="s">
         <v>57</v>
@@ -15542,7 +15542,7 @@
         <v>56</v>
       </c>
       <c r="I311" s="18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J311" s="18" t="s">
         <v>57</v>
@@ -15574,7 +15574,7 @@
         <v>56</v>
       </c>
       <c r="I312" s="16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J312" s="16" t="s">
         <v>57</v>
@@ -15606,7 +15606,7 @@
         <v>56</v>
       </c>
       <c r="I313" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J313" s="18" t="s">
         <v>57</v>
@@ -15638,7 +15638,7 @@
         <v>56</v>
       </c>
       <c r="I314" s="16">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J314" s="16" t="s">
         <v>57</v>
@@ -15670,7 +15670,7 @@
         <v>56</v>
       </c>
       <c r="I315" s="18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J315" s="18" t="s">
         <v>57</v>
@@ -15702,7 +15702,7 @@
         <v>56</v>
       </c>
       <c r="I316" s="16">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J316" s="16" t="s">
         <v>57</v>
@@ -15734,7 +15734,7 @@
         <v>56</v>
       </c>
       <c r="I317" s="18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J317" s="18" t="s">
         <v>57</v>
@@ -15766,7 +15766,7 @@
         <v>56</v>
       </c>
       <c r="I318" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J318" s="16" t="s">
         <v>57</v>
@@ -15830,7 +15830,7 @@
         <v>56</v>
       </c>
       <c r="I320" s="16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J320" s="16" t="s">
         <v>57</v>
@@ -15862,7 +15862,7 @@
         <v>56</v>
       </c>
       <c r="I321" s="18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J321" s="18" t="s">
         <v>57</v>
@@ -15926,7 +15926,7 @@
         <v>56</v>
       </c>
       <c r="I323" s="18">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J323" s="18" t="s">
         <v>57</v>
@@ -15958,7 +15958,7 @@
         <v>56</v>
       </c>
       <c r="I324" s="16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J324" s="16" t="s">
         <v>57</v>
@@ -15990,7 +15990,7 @@
         <v>56</v>
       </c>
       <c r="I325" s="18">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J325" s="18" t="s">
         <v>57</v>
@@ -16022,7 +16022,7 @@
         <v>56</v>
       </c>
       <c r="I326" s="16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J326" s="16" t="s">
         <v>57</v>
@@ -16054,7 +16054,7 @@
         <v>56</v>
       </c>
       <c r="I327" s="18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J327" s="18" t="s">
         <v>57</v>
@@ -16086,7 +16086,7 @@
         <v>56</v>
       </c>
       <c r="I328" s="16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J328" s="16" t="s">
         <v>57</v>
@@ -16118,7 +16118,7 @@
         <v>56</v>
       </c>
       <c r="I329" s="18">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J329" s="18" t="s">
         <v>57</v>
@@ -16150,7 +16150,7 @@
         <v>56</v>
       </c>
       <c r="I330" s="16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J330" s="16" t="s">
         <v>57</v>
@@ -16214,7 +16214,7 @@
         <v>56</v>
       </c>
       <c r="I332" s="16">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J332" s="16" t="s">
         <v>57</v>
@@ -16246,7 +16246,7 @@
         <v>56</v>
       </c>
       <c r="I333" s="18">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J333" s="18" t="s">
         <v>57</v>
@@ -16278,7 +16278,7 @@
         <v>56</v>
       </c>
       <c r="I334" s="16">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J334" s="16" t="s">
         <v>57</v>
@@ -16310,7 +16310,7 @@
         <v>56</v>
       </c>
       <c r="I335" s="18">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J335" s="18" t="s">
         <v>57</v>
@@ -16342,7 +16342,7 @@
         <v>56</v>
       </c>
       <c r="I336" s="16">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J336" s="16" t="s">
         <v>57</v>

</xml_diff>